<commit_message>
Exp3: MI-SAT re-score (goal-agnostic wording) + backlog #7 done
- Re-scored MI-SAT for all 2,784 conversations under the corrected goal-agnostic
  wording (was hard-coded to "diabetes"; personas are smoking/obesity).
  0 errors. Means rise uniformly ~+0.14 vs the old wording (which rated an
  intervention that never happened); all relative conclusions preserved
  (PTO_LA0 still leads, trajectories still climb).
- Re-rendered all 3 views (all/L0/L5), no failures.
- CLAUDE.md: 2026-07-07 landed note + backlog #7 marked done.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Exp3_PTO_GRPO/eda/results/L0/tables/1_outcomes/1_outcomes.xlsx
+++ b/Exp3_PTO_GRPO/eda/results/L0/tables/1_outcomes/1_outcomes.xlsx
@@ -497,7 +497,7 @@
         <v>2.945</v>
       </c>
       <c r="F2" t="n">
-        <v>3.536</v>
+        <v>3.653</v>
       </c>
       <c r="G2" t="n">
         <v>4.273</v>
@@ -537,7 +537,7 @@
         <v>2.749</v>
       </c>
       <c r="F3" t="n">
-        <v>3.326</v>
+        <v>3.441</v>
       </c>
       <c r="G3" t="n">
         <v>4.234</v>

</xml_diff>